<commit_message>
feat: adiciona seção Trabalhos Submetidos
</commit_message>
<xml_diff>
--- a/api/data/examples/eventos.xlsx
+++ b/api/data/examples/eventos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bibianadibellacostabatista/Documents/Thais/Igen/intranet-pasta/projeto-intranet/api/data/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440643C0-6D16-5C4D-A654-A45E9B73538A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D2A198-0E34-AD4F-A59D-DF87D73C485B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="1000" windowWidth="27840" windowHeight="16340" xr2:uid="{6201E4D8-F5B0-AA41-9DF5-65B9990920B6}"/>
+    <workbookView xWindow="29700" yWindow="500" windowWidth="22320" windowHeight="15840" xr2:uid="{6201E4D8-F5B0-AA41-9DF5-65B9990920B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>Data</t>
   </si>
@@ -77,7 +77,64 @@
     <t>Submissão</t>
   </si>
   <si>
-    <t>https://www.atcmeeting.org/Learn/Calls-for-Content/Abstract-Program</t>
+    <t>EFI/BSHI Conference 2026</t>
+  </si>
+  <si>
+    <t>21 a 24/04/26</t>
+  </si>
+  <si>
+    <t>Edimburgo, Escócia</t>
+  </si>
+  <si>
+    <t>19 a 22/08/26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salvador, Brasil </t>
+  </si>
+  <si>
+    <t>XXX Congresso Brasileiro de Terapia Celular e Transplante de Medula Óssea</t>
+  </si>
+  <si>
+    <t>https://congressosbtmo.org.br</t>
+  </si>
+  <si>
+    <t>20 a 23/09/26</t>
+  </si>
+  <si>
+    <t>Sidney, Austrália</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31º Congresso intenacional da Sociedade de Transplantes </t>
+  </si>
+  <si>
+    <t>https://tts2026.org/</t>
+  </si>
+  <si>
+    <t>26 a 30/10/26</t>
+  </si>
+  <si>
+    <t>Montreal, Canadá</t>
+  </si>
+  <si>
+    <t>https://ashi52ndannualmeeting.eventscribe.net/index.asp</t>
+  </si>
+  <si>
+    <t>52º Congresso Anual</t>
+  </si>
+  <si>
+    <t>30/09 a 02/10/26</t>
+  </si>
+  <si>
+    <t>XVIII Congresso Português de Transplantação</t>
+  </si>
+  <si>
+    <t>XXIV Congresso Congresso Luso Brasileiro de Transplantação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coimbra, Portugal </t>
+  </si>
+  <si>
+    <t>https://spt.pt/</t>
   </si>
 </sst>
 </file>
@@ -109,7 +166,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -117,15 +174,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -461,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7B5164B-DE18-DF49-B1DC-3E015A8D83F8}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -490,39 +565,121 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>13</v>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1" xr:uid="{0D282B20-E8C3-BB4D-9210-E0C7086500AC}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{160BF433-F5C2-4547-AD71-A7D9072E1623}"/>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{0D282B20-E8C3-BB4D-9210-E0C7086500AC}"/>
+    <hyperlink ref="D6" r:id="rId2" xr:uid="{B8DDE4E6-EB45-0E42-AB68-AE2968F082A0}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>